<commit_message>
Clarify Google account use for teachers
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="1" r:id="R06b4c2516cf24147"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="學校基本資料" sheetId="2" r:id="R418f4f2f78bd4735"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="班級" sheetId="3" r:id="Raa87409095ae463c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師與配課" sheetId="4" r:id="R49c84c45c634437f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="場地" sheetId="5" r:id="R5e6be1610e254c2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="科目節數" sheetId="6" r:id="Rcfa6975102354910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="年段時段" sheetId="7" r:id="Rf921048aa6094663"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本土語分組" sheetId="8" r:id="R1a313eb871fc4af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="1" r:id="R4d78dc03d8dd46ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="學校基本資料" sheetId="2" r:id="R598e60f6b3f9497b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="班級" sheetId="3" r:id="R05f694d7eab64b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師與配課" sheetId="4" r:id="R849169b6bef14e44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="場地" sheetId="5" r:id="Rdfd505fe3c1f4932"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="科目節數" sheetId="6" r:id="Re8f10cd1af8d44aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="年段時段" sheetId="7" r:id="R952654033083477f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本土語分組" sheetId="8" r:id="R232dda476e064651"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -648,157 +648,209 @@
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="8" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="H9" s="10" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="11" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="G10" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
       <x:c r="H10" s="13" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>學校 Google 帳號用於課表登入：發布課表後，導師可調整負責班級；科任與資源班教師可查看個人課表。只填帳號，不需提供密碼。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="8" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="11" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="G12" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="H12" s="13" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="8" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="F13" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="G13" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="H13" s="10" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="11" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="G14" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="H14" s="13" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="25" customHeight="1">
+      <x:c r="A15" s="8" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="B14" s="12" t="str">
+      <x:c r="B15" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="C14" s="12" t="str">
+      <x:c r="C15" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="D14" s="12" t="str">
+      <x:c r="D15" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="E14" s="12" t="str">
+      <x:c r="E15" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="F14" s="12" t="str">
+      <x:c r="F15" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="G14" s="12" t="str">
+      <x:c r="G15" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="H14" s="13" t="str">
+      <x:c r="H15" s="10" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="25" customHeight="1">
+      <x:c r="A16" s="11" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="G16" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="H16" s="13" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
     </x:row>
@@ -811,6 +863,7 @@
     <x:mergeCell ref="A9:H10"/>
     <x:mergeCell ref="A11:H12"/>
     <x:mergeCell ref="A13:H14"/>
+    <x:mergeCell ref="A15:H16"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1291,25 +1344,25 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="38" t="str">
-        <x:v>教師名冊（導師由班級分頁自動帶入）</x:v>
+        <x:v>教師名冊（學校 Google 帳號供教師登入課表使用）</x:v>
       </x:c>
       <x:c r="B1" s="38" t="str">
-        <x:v>教師名冊（導師由班級分頁自動帶入）</x:v>
+        <x:v>教師名冊（學校 Google 帳號供教師登入課表使用）</x:v>
       </x:c>
       <x:c r="C1" s="38" t="str">
-        <x:v>教師名冊（導師由班級分頁自動帶入）</x:v>
+        <x:v>教師名冊（學校 Google 帳號供教師登入課表使用）</x:v>
       </x:c>
       <x:c r="D1" s="38" t="str">
-        <x:v>教師名冊（導師由班級分頁自動帶入）</x:v>
+        <x:v>教師名冊（學校 Google 帳號供教師登入課表使用）</x:v>
       </x:c>
       <x:c r="E1" s="38" t="str">
-        <x:v>教師名冊（導師由班級分頁自動帶入）</x:v>
+        <x:v>教師名冊（學校 Google 帳號供教師登入課表使用）</x:v>
       </x:c>
       <x:c r="F1" s="38" t="str">
-        <x:v>教師名冊（導師由班級分頁自動帶入）</x:v>
+        <x:v>教師名冊（學校 Google 帳號供教師登入課表使用）</x:v>
       </x:c>
       <x:c r="G1" s="38" t="str">
-        <x:v>教師名冊（導師由班級分頁自動帶入）</x:v>
+        <x:v>教師名冊（學校 Google 帳號供教師登入課表使用）</x:v>
       </x:c>
       <x:c r="H1" s="25"/>
       <x:c r="I1" s="38" t="str">
@@ -1337,7 +1390,8 @@
         <x:v>減課節數</x:v>
       </x:c>
       <x:c r="E2" s="30" t="str">
-        <x:v>Google帳號</x:v>
+        <x:v>學校 Google 帳號
+(課表登入用)</x:v>
       </x:c>
       <x:c r="F2" s="30" t="str">
         <x:v>本土語專長</x:v>

</xml_diff>

<commit_message>
Improve native language teacher setup
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="1" r:id="R4d78dc03d8dd46ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="學校基本資料" sheetId="2" r:id="R598e60f6b3f9497b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="班級" sheetId="3" r:id="R05f694d7eab64b7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師與配課" sheetId="4" r:id="R849169b6bef14e44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="場地" sheetId="5" r:id="Rdfd505fe3c1f4932"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="科目節數" sheetId="6" r:id="Re8f10cd1af8d44aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="年段時段" sheetId="7" r:id="R952654033083477f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本土語分組" sheetId="8" r:id="R232dda476e064651"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="1" r:id="R6c575b3967014ced"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="學校基本資料" sheetId="2" r:id="R12995bd159c441d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="班級" sheetId="3" r:id="R407a8e0f26e94a43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教師與配課" sheetId="4" r:id="R14aeef9ea00f464e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="場地" sheetId="5" r:id="R5ab1e0f587b64759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="科目節數" sheetId="6" r:id="Rc8d42b670afe4f54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="年段時段" sheetId="7" r:id="R0bcb77a6cde34f78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本土語分組" sheetId="8" r:id="R77f631627f384f57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -700,157 +700,209 @@
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="8" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="11" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="G12" s="12" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
       <x:c r="H12" s="13" t="str">
-        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
+        <x:v>教師身分與可授本土語別分開填寫：導師、行政、科任或教支人員都能教授本土語；可授語別可用頓號填多項，教支人員若不需登入可不填 Google 帳號。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="8" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="F13" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="G13" s="9" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="H13" s="10" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="11" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="G14" s="12" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
       <x:c r="H14" s="13" t="str">
-        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+        <x:v>任教班級可填「全部」、「3年級全部」或「3甲、3乙」。多個範圍以頓號或逗號分隔。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="8" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="F15" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="G15" s="9" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
       <x:c r="H15" s="10" t="str">
-        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="11" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="G16" s="12" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+      <x:c r="H16" s="13" t="str">
+        <x:v>灰色／藍色文字為範例資料，請改成貴校內容。標題含 ▾ 的欄位可使用下拉選單，也可以直接輸入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="25" customHeight="1">
+      <x:c r="A17" s="8" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="B16" s="12" t="str">
+      <x:c r="B17" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="C16" s="12" t="str">
+      <x:c r="C17" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="D16" s="12" t="str">
+      <x:c r="D17" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="E16" s="12" t="str">
+      <x:c r="E17" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="F16" s="12" t="str">
+      <x:c r="F17" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="G16" s="12" t="str">
+      <x:c r="G17" s="9" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
-      <x:c r="H16" s="13" t="str">
+      <x:c r="H17" s="10" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="25" customHeight="1">
+      <x:c r="A18" s="11" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="E18" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="F18" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="G18" s="12" t="str">
+        <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
+      </x:c>
+      <x:c r="H18" s="13" t="str">
         <x:v>填寫完成後先在 Excel 儲存，再回到智慧排課系統按「從 Excel 匯入」。上傳後請到配課檢核查看缺配與教師節數。</x:v>
       </x:c>
     </x:row>
@@ -864,6 +916,7 @@
     <x:mergeCell ref="A11:H12"/>
     <x:mergeCell ref="A13:H14"/>
     <x:mergeCell ref="A15:H16"/>
+    <x:mergeCell ref="A17:H18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1334,7 +1387,7 @@
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="4" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
@@ -1380,7 +1433,7 @@
         <x:v>姓名</x:v>
       </x:c>
       <x:c r="B2" s="30" t="str">
-        <x:v>身份 ▾</x:v>
+        <x:v>身分 ▾</x:v>
       </x:c>
       <x:c r="C2" s="30" t="str">
         <x:v>每週節數上限
@@ -1391,10 +1444,11 @@
       </x:c>
       <x:c r="E2" s="30" t="str">
         <x:v>學校 Google 帳號
-(課表登入用)</x:v>
+(教支人員可選填)</x:v>
       </x:c>
       <x:c r="F2" s="30" t="str">
-        <x:v>本土語專長</x:v>
+        <x:v>可授本土語別
+(可複選)</x:v>
       </x:c>
       <x:c r="G2" s="30" t="str">
         <x:v>備註</x:v>
@@ -1517,7 +1571,7 @@
         <x:v>閩語教支</x:v>
       </x:c>
       <x:c r="B7" s="35" t="str">
-        <x:v>鐘點教師</x:v>
+        <x:v>教支人員</x:v>
       </x:c>
       <x:c r="C7" s="35"/>
       <x:c r="D7" s="35" t="n">
@@ -1540,7 +1594,7 @@
         <x:v>客語教支</x:v>
       </x:c>
       <x:c r="B8" s="35" t="str">
-        <x:v>鐘點教師</x:v>
+        <x:v>教支人員</x:v>
       </x:c>
       <x:c r="C8" s="35"/>
       <x:c r="D8" s="35" t="n">
@@ -1563,7 +1617,7 @@
         <x:v>直播教師</x:v>
       </x:c>
       <x:c r="B9" s="35" t="str">
-        <x:v>鐘點教師</x:v>
+        <x:v>教支人員</x:v>
       </x:c>
       <x:c r="C9" s="35"/>
       <x:c r="D9" s="35" t="n">
@@ -2779,7 +2833,7 @@
   </x:mergeCells>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="B3:B100">
-      <x:formula1>"導師,科任,組長,主任,資源班教師,鐘點教師,其他"</x:formula1>
+      <x:formula1>"導師,科任,組長,主任,資源班教師,教支人員,鐘點教師,其他"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J3:J100">
       <x:formula1>"國語文,本土語文,英語文,數學,生活課程,社會,自然科學,音樂,視覺藝術,綜合活動,健康,體育,校訂A,校訂B,校訂C,校訂D,校訂E,校訂F"</x:formula1>
@@ -4789,12 +4843,12 @@
     <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="27" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="25" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="19" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -4812,22 +4866,22 @@
         <x:v>語別</x:v>
       </x:c>
       <x:c r="E1" s="30" t="str">
+        <x:v>分組名稱</x:v>
+      </x:c>
+      <x:c r="F1" s="30" t="str">
+        <x:v>來源班級</x:v>
+      </x:c>
+      <x:c r="G1" s="30" t="str">
+        <x:v>學生人數</x:v>
+      </x:c>
+      <x:c r="H1" s="30" t="str">
         <x:v>授課教師</x:v>
       </x:c>
-      <x:c r="F1" s="30" t="str">
+      <x:c r="I1" s="30" t="str">
+        <x:v>協同教師(選填)</x:v>
+      </x:c>
+      <x:c r="J1" s="30" t="str">
         <x:v>教室 ▾</x:v>
-      </x:c>
-      <x:c r="G1" s="30" t="str">
-        <x:v>協同教師(選填)</x:v>
-      </x:c>
-      <x:c r="H1" s="30" t="str">
-        <x:v>分組名稱</x:v>
-      </x:c>
-      <x:c r="I1" s="30" t="str">
-        <x:v>來源班級</x:v>
-      </x:c>
-      <x:c r="J1" s="30" t="str">
-        <x:v>學生人數</x:v>
       </x:c>
       <x:c r="K1" s="30" t="str">
         <x:v>上課方式</x:v>
@@ -4847,20 +4901,20 @@
         <x:v>閩南語</x:v>
       </x:c>
       <x:c r="E2" s="35" t="str">
+        <x:v>1年級閩南語組</x:v>
+      </x:c>
+      <x:c r="F2" s="35" t="str">
+        <x:v>1甲、1乙</x:v>
+      </x:c>
+      <x:c r="G2" s="35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H2" s="35" t="str">
         <x:v>閩語教支</x:v>
       </x:c>
-      <x:c r="F2" s="35" t="str">
+      <x:c r="I2" s="35"/>
+      <x:c r="J2" s="35" t="str">
         <x:v>原班教室</x:v>
-      </x:c>
-      <x:c r="G2" s="35"/>
-      <x:c r="H2" s="35" t="str">
-        <x:v>1年級閩南語組</x:v>
-      </x:c>
-      <x:c r="I2" s="35" t="str">
-        <x:v>1甲、1乙</x:v>
-      </x:c>
-      <x:c r="J2" s="35" t="n">
-        <x:v>0</x:v>
       </x:c>
       <x:c r="K2" s="35" t="str">
         <x:v>實體</x:v>
@@ -4880,20 +4934,20 @@
         <x:v>客語-四縣</x:v>
       </x:c>
       <x:c r="E3" s="35" t="str">
+        <x:v>1年級客語-四縣組</x:v>
+      </x:c>
+      <x:c r="F3" s="35" t="str">
+        <x:v>1甲、1乙</x:v>
+      </x:c>
+      <x:c r="G3" s="35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H3" s="35" t="str">
         <x:v>客語教支</x:v>
       </x:c>
-      <x:c r="F3" s="35" t="str">
+      <x:c r="I3" s="35"/>
+      <x:c r="J3" s="35" t="str">
         <x:v>英語教室</x:v>
-      </x:c>
-      <x:c r="G3" s="35"/>
-      <x:c r="H3" s="35" t="str">
-        <x:v>1年級客語-四縣組</x:v>
-      </x:c>
-      <x:c r="I3" s="35" t="str">
-        <x:v>1甲、1乙</x:v>
-      </x:c>
-      <x:c r="J3" s="35" t="n">
-        <x:v>0</x:v>
       </x:c>
       <x:c r="K3" s="35" t="str">
         <x:v>實體</x:v>
@@ -4913,22 +4967,22 @@
         <x:v>原民語(直播)</x:v>
       </x:c>
       <x:c r="E4" s="35" t="str">
+        <x:v>1年級原民語(直播)組</x:v>
+      </x:c>
+      <x:c r="F4" s="35" t="str">
+        <x:v>1甲、1乙</x:v>
+      </x:c>
+      <x:c r="G4" s="35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="35" t="str">
         <x:v>直播教師</x:v>
       </x:c>
-      <x:c r="F4" s="35" t="str">
+      <x:c r="I4" s="35" t="str">
+        <x:v>協同人員</x:v>
+      </x:c>
+      <x:c r="J4" s="35" t="str">
         <x:v>電腦教室</x:v>
-      </x:c>
-      <x:c r="G4" s="35" t="str">
-        <x:v>協同人員</x:v>
-      </x:c>
-      <x:c r="H4" s="35" t="str">
-        <x:v>1年級原民語(直播)組</x:v>
-      </x:c>
-      <x:c r="I4" s="35" t="str">
-        <x:v>1甲、1乙</x:v>
-      </x:c>
-      <x:c r="J4" s="35" t="n">
-        <x:v>0</x:v>
       </x:c>
       <x:c r="K4" s="35" t="str">
         <x:v>直播共學</x:v>

</xml_diff>